<commit_message>
focus: adult only mapping of CDE's
</commit_message>
<xml_diff>
--- a/C2D2_docs/c2d2_adult_data_dictionary.xlsx
+++ b/C2D2_docs/c2d2_adult_data_dictionary.xlsx
@@ -2439,7 +2439,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>icu_any_dx_ overdose_withdrawal</t>
+          <t>icu_any_dx_overdose_withdrawal</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">hosp_admit_source </t>
+          <t>hosp_admit_source</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>icu_24hr_any_blood product</t>
+          <t>icu_24hr_any_blood_product</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>icu_24hr_temp_max</t>
+          <t>icu_24hr_temp_min</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -11867,7 +11867,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>icu_24hr_rass_max</t>
+          <t>icu_24hr_rass_min</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">

</xml_diff>